<commit_message>
Rezago matriculados nacional con el formato de 6 a 21, nombres de dos indicadores de Ingresos y correlaciones con Movilidad interna comunal
</commit_message>
<xml_diff>
--- a/output/graficos_dimensiones/comunal_i_peringr_median_a_2018_antofagasta.xlsx
+++ b/output/graficos_dimensiones/comunal_i_peringr_median_a_2018_antofagasta.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
   <si>
     <t xml:space="preserve">Región</t>
   </si>
@@ -69,7 +69,7 @@
     <t xml:space="preserve">Fecha de creación</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-09-23 12:44</t>
+    <t xml:space="preserve">2026-10-01 23:02</t>
   </si>
   <si>
     <t xml:space="preserve">Fuente</t>
@@ -87,7 +87,7 @@
     <t xml:space="preserve">Indicador</t>
   </si>
   <si>
-    <t xml:space="preserve">Ingreso sobre la mediana nacional (%)</t>
+    <t xml:space="preserve">% bajo 50% de la mediana</t>
   </si>
   <si>
     <t xml:space="preserve">Unidad territorial</t>
@@ -100,9 +100,6 @@
   </si>
   <si>
     <t xml:space="preserve">Unidad de medida</t>
-  </si>
-  <si>
-    <t xml:space="preserve">% sobre mediana</t>
   </si>
 </sst>
 </file>
@@ -715,7 +712,7 @@
         <v>27</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>